<commit_message>
Fecha y Hora Inicio/Fin H.E. ahora provienen EXCLUSIVAMENTE de marcaciones biometricas explicitas (Inicio de horas extra / Fin de horas extra)
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_Procesado_Nuevo.xlsx
+++ b/Reporte_Asistencia_Procesado_Nuevo.xlsx
@@ -709,22 +709,22 @@
       </c>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N5" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t>20:17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q5" s="6" t="inlineStr">
@@ -826,22 +826,22 @@
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N6" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P6" s="6" t="inlineStr">
         <is>
-          <t>20:17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q6" s="6" t="inlineStr">
@@ -1052,22 +1052,22 @@
       </c>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P8" s="6" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q8" s="6" t="inlineStr">
@@ -1165,22 +1165,22 @@
       </c>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P9" s="6" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q9" s="6" t="inlineStr">
@@ -1282,22 +1282,22 @@
       </c>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P10" s="6" t="inlineStr">
         <is>
-          <t>19:10</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q10" s="6" t="inlineStr">
@@ -1395,22 +1395,22 @@
       </c>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P11" s="6" t="inlineStr">
         <is>
-          <t>19:10</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q11" s="6" t="inlineStr">
@@ -1512,22 +1512,22 @@
       </c>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N12" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O12" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P12" s="6" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q12" s="6" t="inlineStr">
@@ -1629,22 +1629,22 @@
       </c>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P13" s="6" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q13" s="6" t="inlineStr">
@@ -2073,22 +2073,22 @@
       </c>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O17" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P17" s="6" t="inlineStr">
         <is>
-          <t>07:01</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q17" s="6" t="inlineStr">
@@ -2190,22 +2190,22 @@
       </c>
       <c r="M18" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P18" s="6" t="inlineStr">
         <is>
-          <t>19:01</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q18" s="6" t="inlineStr">
@@ -2303,22 +2303,22 @@
       </c>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P19" s="6" t="inlineStr">
         <is>
-          <t>19:01</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q19" s="6" t="inlineStr">
@@ -2529,22 +2529,22 @@
       </c>
       <c r="M21" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P21" s="6" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q21" s="6" t="inlineStr">
@@ -2642,22 +2642,22 @@
       </c>
       <c r="M22" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N22" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P22" s="6" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q22" s="6" t="inlineStr">
@@ -2759,22 +2759,22 @@
       </c>
       <c r="M23" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N23" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O23" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P23" s="6" t="inlineStr">
         <is>
-          <t>19:02</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q23" s="6" t="inlineStr">
@@ -2872,22 +2872,22 @@
       </c>
       <c r="M24" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O24" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P24" s="6" t="inlineStr">
         <is>
-          <t>19:02</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q24" s="6" t="inlineStr">
@@ -2989,22 +2989,22 @@
       </c>
       <c r="M25" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N25" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O25" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P25" s="6" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q25" s="6" t="inlineStr">
@@ -3102,22 +3102,22 @@
       </c>
       <c r="M26" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N26" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P26" s="6" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q26" s="6" t="inlineStr">
@@ -3219,22 +3219,22 @@
       </c>
       <c r="M27" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N27" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q27" s="6" t="inlineStr">
@@ -3332,22 +3332,22 @@
       </c>
       <c r="M28" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P28" s="6" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q28" s="6" t="inlineStr">
@@ -3449,22 +3449,22 @@
       </c>
       <c r="M29" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N29" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P29" s="6" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr">
@@ -3562,22 +3562,22 @@
       </c>
       <c r="M30" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N30" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P30" s="6" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q30" s="6" t="inlineStr">
@@ -3679,22 +3679,22 @@
       </c>
       <c r="M31" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N31" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P31" s="6" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q31" s="6" t="inlineStr">
@@ -3796,22 +3796,22 @@
       </c>
       <c r="M32" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N32" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P32" s="6" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q32" s="6" t="inlineStr">
@@ -4236,22 +4236,22 @@
       </c>
       <c r="M36" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N36" s="6" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O36" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P36" s="6" t="inlineStr">
         <is>
-          <t>07:01</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q36" s="6" t="inlineStr">
@@ -4349,22 +4349,22 @@
       </c>
       <c r="M37" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N37" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O37" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P37" s="6" t="inlineStr">
         <is>
-          <t>20:18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q37" s="6" t="inlineStr">
@@ -4466,22 +4466,22 @@
       </c>
       <c r="M38" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N38" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O38" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P38" s="6" t="inlineStr">
         <is>
-          <t>20:18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q38" s="6" t="inlineStr">
@@ -4692,22 +4692,22 @@
       </c>
       <c r="M40" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N40" s="6" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O40" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P40" s="6" t="inlineStr">
         <is>
-          <t>07:01</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q40" s="6" t="inlineStr">
@@ -4914,22 +4914,22 @@
       </c>
       <c r="M42" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N42" s="6" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O42" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P42" s="6" t="inlineStr">
         <is>
-          <t>07:06</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q42" s="6" t="inlineStr">
@@ -6153,22 +6153,22 @@
       </c>
       <c r="M53" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N53" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O53" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P53" s="6" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q53" s="6" t="inlineStr">
@@ -6266,22 +6266,22 @@
       </c>
       <c r="M54" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N54" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O54" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P54" s="6" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q54" s="6" t="inlineStr">
@@ -6492,22 +6492,22 @@
       </c>
       <c r="M56" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N56" s="6" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O56" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P56" s="6" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q56" s="6" t="inlineStr">
@@ -6605,22 +6605,22 @@
       </c>
       <c r="M57" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N57" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O57" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P57" s="6" t="inlineStr">
         <is>
-          <t>19:03</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q57" s="6" t="inlineStr">
@@ -6718,22 +6718,22 @@
       </c>
       <c r="M58" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N58" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O58" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P58" s="6" t="inlineStr">
         <is>
-          <t>19:03</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q58" s="6" t="inlineStr">
@@ -6835,22 +6835,22 @@
       </c>
       <c r="M59" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N59" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O59" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P59" s="6" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q59" s="6" t="inlineStr">
@@ -6948,22 +6948,22 @@
       </c>
       <c r="M60" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N60" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O60" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P60" s="6" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q60" s="6" t="inlineStr">
@@ -7065,22 +7065,22 @@
       </c>
       <c r="M61" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N61" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O61" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P61" s="6" t="inlineStr">
         <is>
-          <t>19:13</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q61" s="6" t="inlineStr">
@@ -7182,22 +7182,22 @@
       </c>
       <c r="M62" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N62" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O62" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P62" s="6" t="inlineStr">
         <is>
-          <t>19:13</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q62" s="6" t="inlineStr">
@@ -7299,22 +7299,22 @@
       </c>
       <c r="M63" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N63" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O63" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P63" s="6" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q63" s="6" t="inlineStr">
@@ -7412,22 +7412,22 @@
       </c>
       <c r="M64" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N64" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O64" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P64" s="6" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q64" s="6" t="inlineStr">
@@ -7763,22 +7763,22 @@
       </c>
       <c r="M67" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N67" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O67" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P67" s="6" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q67" s="6" t="inlineStr">
@@ -7876,22 +7876,22 @@
       </c>
       <c r="M68" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N68" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O68" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P68" s="6" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q68" s="6" t="inlineStr">
@@ -7993,22 +7993,22 @@
       </c>
       <c r="M69" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N69" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O69" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P69" s="6" t="inlineStr">
         <is>
-          <t>19:13</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q69" s="6" t="inlineStr">
@@ -8106,22 +8106,22 @@
       </c>
       <c r="M70" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N70" s="6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O70" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P70" s="6" t="inlineStr">
         <is>
-          <t>19:13</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q70" s="6" t="inlineStr">
@@ -9006,22 +9006,22 @@
       </c>
       <c r="M78" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N78" s="6" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O78" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P78" s="6" t="inlineStr">
         <is>
-          <t>07:06</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q78" s="6" t="inlineStr">

</xml_diff>